<commit_message>
Implement production readiness, UI, safety, and privacy pass
</commit_message>
<xml_diff>
--- a/templates/beeline_archive.template.xlsx
+++ b/templates/beeline_archive.template.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03T14:40:30+00:00</t>
+          <t>2026-06-03T15:51:40+00:00</t>
         </is>
       </c>
     </row>
@@ -581,10 +581,22 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Grouped refresh</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Archive writer</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>openpyxl, no Excel COM required</t>
         </is>
@@ -725,7 +737,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Newest resolved dates are shown first. Updated 2026-06-03T14:40:30+00:00.</t>
+          <t>Newest resolved dates are shown first. Updated 2026-06-03T15:51:40+00:00.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement local predictive maintenance analytics
</commit_message>
<xml_diff>
--- a/templates/beeline_archive.template.xlsx
+++ b/templates/beeline_archive.template.xlsx
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03T15:51:40+00:00</t>
+          <t>2026-06-03T16:25:07+00:00</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Newest resolved dates are shown first. Updated 2026-06-03T15:51:40+00:00.</t>
+          <t>Newest resolved dates are shown first. Updated 2026-06-03T16:25:07+00:00.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement BeeLine performance and archive search architecture
</commit_message>
<xml_diff>
--- a/templates/beeline_archive.template.xlsx
+++ b/templates/beeline_archive.template.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resolved_By_Date" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resolved_Issues'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resolved_Issues'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resolved_By_Date'!$A$3:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03T16:25:07+00:00</t>
+          <t>2026-06-03T18:14:16+00:00</t>
         </is>
       </c>
     </row>
@@ -617,21 +617,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -647,57 +648,62 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
+          <t>issue_id</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
           <t>machine_number</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>logged_by</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>created_at_utc</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>resolved_at_utc</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>resolved_by</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>solution</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -712,7 +718,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
@@ -737,7 +743,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Newest resolved dates are shown first. Updated 2026-06-03T16:25:07+00:00.</t>
+          <t>Newest resolved dates are shown first. Updated 2026-06-03T18:14:16+00:00.</t>
         </is>
       </c>
     </row>

</xml_diff>